<commit_message>
Update chip report site 2026-05-14
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-04-22.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-04-22.xlsx
@@ -114,7 +114,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -136,11 +136,104 @@
         <color rgb="00c7d6e5"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00c7d6e5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00c7d6e5"/>
+      </right>
+      <top style="thin">
+        <color rgb="00c7d6e5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00c7d6e5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00c7d6e5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00c7d6e5"/>
+      </right>
+      <top style="thin">
+        <color rgb="00c7d6e5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00c7d6e5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00c7d6e5"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00c7d6e5"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00c7d6e5"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00c7d6e5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00c7d6e5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00c7d6e5"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00c7d6e5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -188,6 +281,13 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -586,25 +686,26 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>留倉概況</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
+      <c r="B4" s="17" t="n"/>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="17" t="n"/>
+      <c r="M4" s="17" t="n"/>
+      <c r="N4" s="18" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -612,22 +713,22 @@
           <t>日期</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
+      <c r="B5" s="17" t="n"/>
+      <c r="C5" s="18" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>結算日</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="18" t="n"/>
       <c r="I5" s="5" t="inlineStr">
         <is>
           <t>當次月大台留倉差增減</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -635,29 +736,29 @@
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="20" t="n"/>
       <c r="E6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="20" t="n"/>
       <c r="I6" s="6" t="n">
         <v>-926</v>
       </c>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
+      <c r="J6" s="19" t="n"/>
+      <c r="K6" s="20" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="6" t="n"/>
+      <c r="A7" s="21" t="n"/>
+      <c r="B7" s="22" t="n"/>
+      <c r="C7" s="23" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="23" t="n"/>
+      <c r="I7" s="21" t="n"/>
+      <c r="J7" s="22" t="n"/>
+      <c r="K7" s="23" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -665,53 +766,55 @@
           <t>今日日盤後整理</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="20" t="n"/>
       <c r="E8" s="7" t="inlineStr">
         <is>
           <t>原表編碼對應星期三</t>
         </is>
       </c>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="20" t="n"/>
       <c r="I8" s="7" t="inlineStr">
         <is>
           <t>(81,421-2,122) - (82,127-1,902)</t>
         </is>
       </c>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="20" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-    </row>
+      <c r="A9" s="21" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="23" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="23" t="n"/>
+      <c r="I9" s="21" t="n"/>
+      <c r="J9" s="22" t="n"/>
+      <c r="K9" s="23" t="n"/>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>大盤資訊</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="n"/>
-      <c r="L12" s="4" t="n"/>
-      <c r="M12" s="4" t="n"/>
-      <c r="N12" s="4" t="n"/>
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="17" t="n"/>
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="17" t="n"/>
+      <c r="J12" s="17" t="n"/>
+      <c r="K12" s="17" t="n"/>
+      <c r="L12" s="17" t="n"/>
+      <c r="M12" s="17" t="n"/>
+      <c r="N12" s="18" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -719,50 +822,50 @@
           <t>加權指數</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
+      <c r="B13" s="17" t="n"/>
+      <c r="C13" s="18" t="n"/>
       <c r="E13" s="9" t="inlineStr">
         <is>
           <t>加權指數漲跌</t>
         </is>
       </c>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
+      <c r="F13" s="17" t="n"/>
+      <c r="G13" s="18" t="n"/>
       <c r="I13" s="9" t="inlineStr">
         <is>
           <t>加權指數漲跌幅(%)</t>
         </is>
       </c>
-      <c r="J13" s="9" t="n"/>
-      <c r="K13" s="9" t="n"/>
+      <c r="J13" s="17" t="n"/>
+      <c r="K13" s="18" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
         <v>37878.47</v>
       </c>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="20" t="n"/>
       <c r="E14" s="6" t="n">
         <v>273.36</v>
       </c>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="20" t="n"/>
       <c r="I14" s="6" t="n">
         <v>0.73</v>
       </c>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="6" t="n"/>
+      <c r="J14" s="19" t="n"/>
+      <c r="K14" s="20" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="6" t="n"/>
+      <c r="A15" s="21" t="n"/>
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="23" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="22" t="n"/>
+      <c r="G15" s="23" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="22" t="n"/>
+      <c r="K15" s="23" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -770,33 +873,33 @@
           <t>TWSE MI_INDEX 收盤數據</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="20" t="n"/>
       <c r="E16" s="7" t="inlineStr">
         <is>
           <t>TWSE MI_INDEX 收盤數據</t>
         </is>
       </c>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="20" t="n"/>
       <c r="I16" s="7" t="inlineStr">
         <is>
           <t>TWSE MI_INDEX 收盤數據</t>
         </is>
       </c>
-      <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="n"/>
+      <c r="J16" s="19" t="n"/>
+      <c r="K16" s="20" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
+      <c r="A17" s="21" t="n"/>
+      <c r="B17" s="22" t="n"/>
+      <c r="C17" s="23" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="22" t="n"/>
+      <c r="G17" s="23" t="n"/>
+      <c r="I17" s="21" t="n"/>
+      <c r="J17" s="22" t="n"/>
+      <c r="K17" s="23" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1"/>
     <row r="19">
@@ -805,50 +908,50 @@
           <t>加權指數當日高低差</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="18" t="n"/>
       <c r="E19" s="9" t="inlineStr">
         <is>
           <t>加權指數成交量(億)</t>
         </is>
       </c>
-      <c r="F19" s="9" t="n"/>
-      <c r="G19" s="9" t="n"/>
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="18" t="n"/>
       <c r="I19" s="9" t="inlineStr">
         <is>
           <t>PCR與結算比</t>
         </is>
       </c>
-      <c r="J19" s="9" t="n"/>
-      <c r="K19" s="9" t="n"/>
+      <c r="J19" s="17" t="n"/>
+      <c r="K19" s="18" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
         <v>473.5</v>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="20" t="n"/>
       <c r="E20" s="6" t="n">
         <v>9798.76044142</v>
       </c>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="20" t="n"/>
       <c r="I20" s="6" t="n">
         <v>139.67</v>
       </c>
-      <c r="J20" s="6" t="n"/>
-      <c r="K20" s="6" t="n"/>
+      <c r="J20" s="19" t="n"/>
+      <c r="K20" s="20" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="I21" s="6" t="n"/>
-      <c r="J21" s="6" t="n"/>
-      <c r="K21" s="6" t="n"/>
+      <c r="A21" s="21" t="n"/>
+      <c r="B21" s="22" t="n"/>
+      <c r="C21" s="23" t="n"/>
+      <c r="E21" s="21" t="n"/>
+      <c r="F21" s="22" t="n"/>
+      <c r="G21" s="23" t="n"/>
+      <c r="I21" s="21" t="n"/>
+      <c r="J21" s="22" t="n"/>
+      <c r="K21" s="23" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -856,84 +959,85 @@
           <t>38,096.88 - 37,623.38；TWSE MI_5MINS_HIST</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="20" t="n"/>
       <c r="E22" s="7" t="inlineStr">
         <is>
           <t>TWSE MI_INDEX 大盤統計資訊總計(億元)</t>
         </is>
       </c>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="20" t="n"/>
       <c r="I22" s="7" t="inlineStr">
         <is>
           <t>TAIFEX pcRatio 2026-04-22</t>
         </is>
       </c>
-      <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
+      <c r="J22" s="19" t="n"/>
+      <c r="K22" s="20" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n"/>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
-    </row>
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="22" t="n"/>
+      <c r="C23" s="23" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="22" t="n"/>
+      <c r="G23" s="23" t="n"/>
+      <c r="I23" s="21" t="n"/>
+      <c r="J23" s="22" t="n"/>
+      <c r="K23" s="23" t="n"/>
+    </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t>融資金額(仟元)</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="n"/>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="18" t="n"/>
       <c r="E25" s="9" t="inlineStr">
         <is>
           <t>融資金額變化量</t>
         </is>
       </c>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="9" t="n"/>
+      <c r="F25" s="17" t="n"/>
+      <c r="G25" s="18" t="n"/>
       <c r="I25" s="9" t="inlineStr">
         <is>
           <t>融券(交易單位)</t>
         </is>
       </c>
-      <c r="J25" s="9" t="n"/>
-      <c r="K25" s="9" t="n"/>
+      <c r="J25" s="17" t="n"/>
+      <c r="K25" s="18" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
         <v>438545241</v>
       </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="20" t="n"/>
       <c r="E26" s="6" t="n">
         <v>5381347</v>
       </c>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="20" t="n"/>
       <c r="I26" s="6" t="n">
         <v>185944</v>
       </c>
-      <c r="J26" s="6" t="n"/>
-      <c r="K26" s="6" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="20" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="J27" s="6" t="n"/>
-      <c r="K27" s="6" t="n"/>
+      <c r="A27" s="21" t="n"/>
+      <c r="B27" s="22" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="22" t="n"/>
+      <c r="G27" s="23" t="n"/>
+      <c r="I27" s="21" t="n"/>
+      <c r="J27" s="22" t="n"/>
+      <c r="K27" s="23" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -941,54 +1045,55 @@
           <t>TWSE MI_MARGN 4/22 今日餘額</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="n"/>
+      <c r="B28" s="19" t="n"/>
+      <c r="C28" s="20" t="n"/>
       <c r="E28" s="7" t="inlineStr">
         <is>
           <t>438,545,241 - 433,163,894</t>
         </is>
       </c>
-      <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="20" t="n"/>
       <c r="I28" s="7" t="inlineStr">
         <is>
           <t>TWSE MI_MARGN 4/22 今日餘額</t>
         </is>
       </c>
-      <c r="J28" s="7" t="n"/>
-      <c r="K28" s="7" t="n"/>
+      <c r="J28" s="19" t="n"/>
+      <c r="K28" s="20" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
-      <c r="F29" s="7" t="n"/>
-      <c r="G29" s="7" t="n"/>
-      <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="n"/>
-    </row>
+      <c r="A29" s="21" t="n"/>
+      <c r="B29" s="22" t="n"/>
+      <c r="C29" s="23" t="n"/>
+      <c r="E29" s="21" t="n"/>
+      <c r="F29" s="22" t="n"/>
+      <c r="G29" s="23" t="n"/>
+      <c r="I29" s="21" t="n"/>
+      <c r="J29" s="22" t="n"/>
+      <c r="K29" s="23" t="n"/>
+    </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
           <t>融券單位變化量</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="18" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="6" t="n">
         <v>-4453</v>
       </c>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="6" t="n"/>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="20" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
+      <c r="A33" s="21" t="n"/>
+      <c r="B33" s="22" t="n"/>
+      <c r="C33" s="23" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -996,33 +1101,35 @@
           <t>185,944 - 190,397</t>
         </is>
       </c>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="20" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n"/>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n"/>
-    </row>
+      <c r="A35" s="21" t="n"/>
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="23" t="n"/>
+    </row>
+    <row r="36"/>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
           <t>外資布局</t>
         </is>
       </c>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
-      <c r="H38" s="4" t="n"/>
-      <c r="I38" s="4" t="n"/>
-      <c r="J38" s="4" t="n"/>
-      <c r="K38" s="4" t="n"/>
-      <c r="L38" s="4" t="n"/>
-      <c r="M38" s="4" t="n"/>
-      <c r="N38" s="4" t="n"/>
+      <c r="B38" s="17" t="n"/>
+      <c r="C38" s="17" t="n"/>
+      <c r="D38" s="17" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17" t="n"/>
+      <c r="G38" s="17" t="n"/>
+      <c r="H38" s="17" t="n"/>
+      <c r="I38" s="17" t="n"/>
+      <c r="J38" s="17" t="n"/>
+      <c r="K38" s="17" t="n"/>
+      <c r="L38" s="17" t="n"/>
+      <c r="M38" s="17" t="n"/>
+      <c r="N38" s="18" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
@@ -1030,50 +1137,50 @@
           <t>外資現貨買賣超</t>
         </is>
       </c>
-      <c r="B39" s="11" t="n"/>
-      <c r="C39" s="11" t="n"/>
+      <c r="B39" s="17" t="n"/>
+      <c r="C39" s="18" t="n"/>
       <c r="E39" s="11" t="inlineStr">
         <is>
           <t>外資(大小台)期貨未平倉</t>
         </is>
       </c>
-      <c r="F39" s="11" t="n"/>
-      <c r="G39" s="11" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="18" t="n"/>
       <c r="I39" s="11" t="inlineStr">
         <is>
           <t>外資期貨未平倉與結算比</t>
         </is>
       </c>
-      <c r="J39" s="11" t="n"/>
-      <c r="K39" s="11" t="n"/>
+      <c r="J39" s="17" t="n"/>
+      <c r="K39" s="18" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
         <v>116.09</v>
       </c>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="20" t="n"/>
       <c r="E40" s="6" t="n">
         <v>-42115</v>
       </c>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="6" t="n"/>
+      <c r="F40" s="19" t="n"/>
+      <c r="G40" s="20" t="n"/>
       <c r="I40" s="6" t="n">
         <v>-5227</v>
       </c>
-      <c r="J40" s="6" t="n"/>
-      <c r="K40" s="6" t="n"/>
+      <c r="J40" s="19" t="n"/>
+      <c r="K40" s="20" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="6" t="n"/>
-      <c r="I41" s="6" t="n"/>
-      <c r="J41" s="6" t="n"/>
-      <c r="K41" s="6" t="n"/>
+      <c r="A41" s="21" t="n"/>
+      <c r="B41" s="22" t="n"/>
+      <c r="C41" s="23" t="n"/>
+      <c r="E41" s="21" t="n"/>
+      <c r="F41" s="22" t="n"/>
+      <c r="G41" s="23" t="n"/>
+      <c r="I41" s="21" t="n"/>
+      <c r="J41" s="22" t="n"/>
+      <c r="K41" s="23" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -1081,33 +1188,33 @@
           <t>TWSE BFI82U 三大法人摘要，億元</t>
         </is>
       </c>
-      <c r="B42" s="7" t="n"/>
-      <c r="C42" s="7" t="n"/>
+      <c r="B42" s="19" t="n"/>
+      <c r="C42" s="20" t="n"/>
       <c r="E42" s="7" t="inlineStr">
         <is>
           <t>TAIFEX 合併口徑 = -42,555 + 1,334/4 + 2,126/20，四捨五入</t>
         </is>
       </c>
-      <c r="F42" s="7" t="n"/>
-      <c r="G42" s="7" t="n"/>
+      <c r="F42" s="19" t="n"/>
+      <c r="G42" s="20" t="n"/>
       <c r="I42" s="7" t="inlineStr">
         <is>
           <t>-42,115.20 - (-36,888) ≈ -5,227</t>
         </is>
       </c>
-      <c r="J42" s="7" t="n"/>
-      <c r="K42" s="7" t="n"/>
+      <c r="J42" s="19" t="n"/>
+      <c r="K42" s="20" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="n"/>
-      <c r="B43" s="7" t="n"/>
-      <c r="C43" s="7" t="n"/>
-      <c r="E43" s="7" t="n"/>
-      <c r="F43" s="7" t="n"/>
-      <c r="G43" s="7" t="n"/>
-      <c r="I43" s="7" t="n"/>
-      <c r="J43" s="7" t="n"/>
-      <c r="K43" s="7" t="n"/>
+      <c r="A43" s="21" t="n"/>
+      <c r="B43" s="22" t="n"/>
+      <c r="C43" s="23" t="n"/>
+      <c r="E43" s="21" t="n"/>
+      <c r="F43" s="22" t="n"/>
+      <c r="G43" s="23" t="n"/>
+      <c r="I43" s="21" t="n"/>
+      <c r="J43" s="22" t="n"/>
+      <c r="K43" s="23" t="n"/>
     </row>
     <row r="44" ht="22" customHeight="1"/>
     <row r="45">
@@ -1116,50 +1223,50 @@
           <t>外資期貨未平倉與前日增減</t>
         </is>
       </c>
-      <c r="B45" s="11" t="n"/>
-      <c r="C45" s="11" t="n"/>
+      <c r="B45" s="17" t="n"/>
+      <c r="C45" s="18" t="n"/>
       <c r="E45" s="11" t="inlineStr">
         <is>
           <t>外資(買)OP未平倉口數</t>
         </is>
       </c>
-      <c r="F45" s="11" t="n"/>
-      <c r="G45" s="11" t="n"/>
+      <c r="F45" s="17" t="n"/>
+      <c r="G45" s="18" t="n"/>
       <c r="I45" s="11" t="inlineStr">
         <is>
           <t>外資(買)OP未平倉金額</t>
         </is>
       </c>
-      <c r="J45" s="11" t="n"/>
-      <c r="K45" s="11" t="n"/>
+      <c r="J45" s="17" t="n"/>
+      <c r="K45" s="18" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
         <v>-2034</v>
       </c>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="6" t="n"/>
+      <c r="B46" s="19" t="n"/>
+      <c r="C46" s="20" t="n"/>
       <c r="E46" s="6" t="n">
         <v>-348</v>
       </c>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="6" t="n"/>
+      <c r="F46" s="19" t="n"/>
+      <c r="G46" s="20" t="n"/>
       <c r="I46" s="6" t="n">
         <v>195694</v>
       </c>
-      <c r="J46" s="6" t="n"/>
-      <c r="K46" s="6" t="n"/>
+      <c r="J46" s="19" t="n"/>
+      <c r="K46" s="20" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="6" t="n"/>
-      <c r="I47" s="6" t="n"/>
-      <c r="J47" s="6" t="n"/>
-      <c r="K47" s="6" t="n"/>
+      <c r="A47" s="21" t="n"/>
+      <c r="B47" s="22" t="n"/>
+      <c r="C47" s="23" t="n"/>
+      <c r="E47" s="21" t="n"/>
+      <c r="F47" s="22" t="n"/>
+      <c r="G47" s="23" t="n"/>
+      <c r="I47" s="21" t="n"/>
+      <c r="J47" s="22" t="n"/>
+      <c r="K47" s="23" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -1167,84 +1274,85 @@
           <t>-42,115.20 - (-40,081) ≈ -2,034</t>
         </is>
       </c>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="7" t="n"/>
+      <c r="B48" s="19" t="n"/>
+      <c r="C48" s="20" t="n"/>
       <c r="E48" s="7" t="inlineStr">
         <is>
           <t>BC - SC / TAIFEX 選擇權買賣權分計</t>
         </is>
       </c>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="7" t="n"/>
+      <c r="F48" s="19" t="n"/>
+      <c r="G48" s="20" t="n"/>
       <c r="I48" s="7" t="inlineStr">
         <is>
           <t>BC金額 - SC金額，仟元</t>
         </is>
       </c>
-      <c r="J48" s="7" t="n"/>
-      <c r="K48" s="7" t="n"/>
+      <c r="J48" s="19" t="n"/>
+      <c r="K48" s="20" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n"/>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="7" t="n"/>
-      <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="n"/>
-      <c r="G49" s="7" t="n"/>
-      <c r="I49" s="7" t="n"/>
-      <c r="J49" s="7" t="n"/>
-      <c r="K49" s="7" t="n"/>
-    </row>
+      <c r="A49" s="21" t="n"/>
+      <c r="B49" s="22" t="n"/>
+      <c r="C49" s="23" t="n"/>
+      <c r="E49" s="21" t="n"/>
+      <c r="F49" s="22" t="n"/>
+      <c r="G49" s="23" t="n"/>
+      <c r="I49" s="21" t="n"/>
+      <c r="J49" s="22" t="n"/>
+      <c r="K49" s="23" t="n"/>
+    </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
           <t>外資(BC)OP未平倉金額與結算比</t>
         </is>
       </c>
-      <c r="B51" s="11" t="n"/>
-      <c r="C51" s="11" t="n"/>
+      <c r="B51" s="17" t="n"/>
+      <c r="C51" s="18" t="n"/>
       <c r="E51" s="11" t="inlineStr">
         <is>
           <t>外資(賣)OP未平倉口數</t>
         </is>
       </c>
-      <c r="F51" s="11" t="n"/>
-      <c r="G51" s="11" t="n"/>
+      <c r="F51" s="17" t="n"/>
+      <c r="G51" s="18" t="n"/>
       <c r="I51" s="11" t="inlineStr">
         <is>
           <t>外資(賣)OP未平倉金額</t>
         </is>
       </c>
-      <c r="J51" s="11" t="n"/>
-      <c r="K51" s="11" t="n"/>
+      <c r="J51" s="17" t="n"/>
+      <c r="K51" s="18" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
         <v>292191</v>
       </c>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="6" t="n"/>
+      <c r="B52" s="19" t="n"/>
+      <c r="C52" s="20" t="n"/>
       <c r="E52" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="6" t="n"/>
+      <c r="F52" s="19" t="n"/>
+      <c r="G52" s="20" t="n"/>
       <c r="I52" s="6" t="n">
         <v>16864</v>
       </c>
-      <c r="J52" s="6" t="n"/>
-      <c r="K52" s="6" t="n"/>
+      <c r="J52" s="19" t="n"/>
+      <c r="K52" s="20" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n"/>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="6" t="n"/>
-      <c r="I53" s="6" t="n"/>
-      <c r="J53" s="6" t="n"/>
-      <c r="K53" s="6" t="n"/>
+      <c r="A53" s="21" t="n"/>
+      <c r="B53" s="22" t="n"/>
+      <c r="C53" s="23" t="n"/>
+      <c r="E53" s="21" t="n"/>
+      <c r="F53" s="22" t="n"/>
+      <c r="G53" s="23" t="n"/>
+      <c r="I53" s="21" t="n"/>
+      <c r="J53" s="22" t="n"/>
+      <c r="K53" s="23" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -1252,84 +1360,85 @@
           <t>1,098,547 - 806,356(4/15結算日 BC 原始金額)</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="7" t="n"/>
+      <c r="B54" s="19" t="n"/>
+      <c r="C54" s="20" t="n"/>
       <c r="E54" s="7" t="inlineStr">
         <is>
           <t>BP - SP / TAIFEX 選擇權買賣權分計</t>
         </is>
       </c>
-      <c r="F54" s="7" t="n"/>
-      <c r="G54" s="7" t="n"/>
+      <c r="F54" s="19" t="n"/>
+      <c r="G54" s="20" t="n"/>
       <c r="I54" s="7" t="inlineStr">
         <is>
           <t>BP金額 - SP金額，仟元</t>
         </is>
       </c>
-      <c r="J54" s="7" t="n"/>
-      <c r="K54" s="7" t="n"/>
+      <c r="J54" s="19" t="n"/>
+      <c r="K54" s="20" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="n"/>
-      <c r="B55" s="7" t="n"/>
-      <c r="C55" s="7" t="n"/>
-      <c r="E55" s="7" t="n"/>
-      <c r="F55" s="7" t="n"/>
-      <c r="G55" s="7" t="n"/>
-      <c r="I55" s="7" t="n"/>
-      <c r="J55" s="7" t="n"/>
-      <c r="K55" s="7" t="n"/>
-    </row>
+      <c r="A55" s="21" t="n"/>
+      <c r="B55" s="22" t="n"/>
+      <c r="C55" s="23" t="n"/>
+      <c r="E55" s="21" t="n"/>
+      <c r="F55" s="22" t="n"/>
+      <c r="G55" s="23" t="n"/>
+      <c r="I55" s="21" t="n"/>
+      <c r="J55" s="22" t="n"/>
+      <c r="K55" s="23" t="n"/>
+    </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
           <t>外資(BP)OP未平倉金額與結算比</t>
         </is>
       </c>
-      <c r="B57" s="11" t="n"/>
-      <c r="C57" s="11" t="n"/>
+      <c r="B57" s="17" t="n"/>
+      <c r="C57" s="18" t="n"/>
       <c r="E57" s="11" t="inlineStr">
         <is>
           <t>外資買方買權/賣權比</t>
         </is>
       </c>
-      <c r="F57" s="11" t="n"/>
-      <c r="G57" s="11" t="n"/>
+      <c r="F57" s="17" t="n"/>
+      <c r="G57" s="18" t="n"/>
       <c r="I57" s="11" t="inlineStr">
         <is>
           <t>外資買權/賣權比</t>
         </is>
       </c>
-      <c r="J57" s="11" t="n"/>
-      <c r="K57" s="11" t="n"/>
+      <c r="J57" s="17" t="n"/>
+      <c r="K57" s="18" t="n"/>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="6" t="n">
         <v>-309</v>
       </c>
-      <c r="B58" s="6" t="n"/>
-      <c r="C58" s="6" t="n"/>
+      <c r="B58" s="19" t="n"/>
+      <c r="C58" s="20" t="n"/>
       <c r="E58" s="6" t="n">
         <v>0.6609170113526357</v>
       </c>
-      <c r="F58" s="6" t="n"/>
-      <c r="G58" s="6" t="n"/>
+      <c r="F58" s="19" t="n"/>
+      <c r="G58" s="20" t="n"/>
       <c r="I58" s="6" t="n">
         <v>0.6762596259625963</v>
       </c>
-      <c r="J58" s="6" t="n"/>
-      <c r="K58" s="6" t="n"/>
+      <c r="J58" s="19" t="n"/>
+      <c r="K58" s="20" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="n"/>
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="6" t="n"/>
-      <c r="E59" s="6" t="n"/>
-      <c r="F59" s="6" t="n"/>
-      <c r="G59" s="6" t="n"/>
-      <c r="I59" s="6" t="n"/>
-      <c r="J59" s="6" t="n"/>
-      <c r="K59" s="6" t="n"/>
+      <c r="A59" s="21" t="n"/>
+      <c r="B59" s="22" t="n"/>
+      <c r="C59" s="23" t="n"/>
+      <c r="E59" s="21" t="n"/>
+      <c r="F59" s="22" t="n"/>
+      <c r="G59" s="23" t="n"/>
+      <c r="I59" s="21" t="n"/>
+      <c r="J59" s="22" t="n"/>
+      <c r="K59" s="23" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -1337,53 +1446,55 @@
           <t>125,723 - 126,032(4/15結算日 BP 原始金額)</t>
         </is>
       </c>
-      <c r="B60" s="7" t="n"/>
-      <c r="C60" s="7" t="n"/>
+      <c r="B60" s="19" t="n"/>
+      <c r="C60" s="20" t="n"/>
       <c r="E60" s="7" t="inlineStr">
         <is>
           <t>7,510 / 11,363</t>
         </is>
       </c>
-      <c r="F60" s="7" t="n"/>
-      <c r="G60" s="7" t="n"/>
+      <c r="F60" s="19" t="n"/>
+      <c r="G60" s="20" t="n"/>
       <c r="I60" s="7" t="inlineStr">
         <is>
           <t>(7,510+7,858) / (11,363+11,362)</t>
         </is>
       </c>
-      <c r="J60" s="7" t="n"/>
-      <c r="K60" s="7" t="n"/>
+      <c r="J60" s="19" t="n"/>
+      <c r="K60" s="20" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="n"/>
-      <c r="B61" s="7" t="n"/>
-      <c r="C61" s="7" t="n"/>
-      <c r="E61" s="7" t="n"/>
-      <c r="F61" s="7" t="n"/>
-      <c r="G61" s="7" t="n"/>
-      <c r="I61" s="7" t="n"/>
-      <c r="J61" s="7" t="n"/>
-      <c r="K61" s="7" t="n"/>
-    </row>
+      <c r="A61" s="21" t="n"/>
+      <c r="B61" s="22" t="n"/>
+      <c r="C61" s="23" t="n"/>
+      <c r="E61" s="21" t="n"/>
+      <c r="F61" s="22" t="n"/>
+      <c r="G61" s="23" t="n"/>
+      <c r="I61" s="21" t="n"/>
+      <c r="J61" s="22" t="n"/>
+      <c r="K61" s="23" t="n"/>
+    </row>
+    <row r="62"/>
+    <row r="63"/>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
         <is>
           <t>自營布局</t>
         </is>
       </c>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="4" t="n"/>
-      <c r="E64" s="4" t="n"/>
-      <c r="F64" s="4" t="n"/>
-      <c r="G64" s="4" t="n"/>
-      <c r="H64" s="4" t="n"/>
-      <c r="I64" s="4" t="n"/>
-      <c r="J64" s="4" t="n"/>
-      <c r="K64" s="4" t="n"/>
-      <c r="L64" s="4" t="n"/>
-      <c r="M64" s="4" t="n"/>
-      <c r="N64" s="4" t="n"/>
+      <c r="B64" s="17" t="n"/>
+      <c r="C64" s="17" t="n"/>
+      <c r="D64" s="17" t="n"/>
+      <c r="E64" s="17" t="n"/>
+      <c r="F64" s="17" t="n"/>
+      <c r="G64" s="17" t="n"/>
+      <c r="H64" s="17" t="n"/>
+      <c r="I64" s="17" t="n"/>
+      <c r="J64" s="17" t="n"/>
+      <c r="K64" s="17" t="n"/>
+      <c r="L64" s="17" t="n"/>
+      <c r="M64" s="17" t="n"/>
+      <c r="N64" s="18" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="13" t="inlineStr">
@@ -1391,50 +1502,50 @@
           <t>自營(自行)現貨買賣超</t>
         </is>
       </c>
-      <c r="B65" s="13" t="n"/>
-      <c r="C65" s="13" t="n"/>
+      <c r="B65" s="17" t="n"/>
+      <c r="C65" s="18" t="n"/>
       <c r="E65" s="13" t="inlineStr">
         <is>
           <t>自營(避險)現貨買賣超</t>
         </is>
       </c>
-      <c r="F65" s="13" t="n"/>
-      <c r="G65" s="13" t="n"/>
+      <c r="F65" s="17" t="n"/>
+      <c r="G65" s="18" t="n"/>
       <c r="I65" s="13" t="inlineStr">
         <is>
           <t>自營(大小台)期貨未平倉</t>
         </is>
       </c>
-      <c r="J65" s="13" t="n"/>
-      <c r="K65" s="13" t="n"/>
+      <c r="J65" s="17" t="n"/>
+      <c r="K65" s="18" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n">
         <v>13.28</v>
       </c>
-      <c r="B66" s="6" t="n"/>
-      <c r="C66" s="6" t="n"/>
+      <c r="B66" s="19" t="n"/>
+      <c r="C66" s="20" t="n"/>
       <c r="E66" s="6" t="n">
         <v>-5.9</v>
       </c>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="6" t="n"/>
+      <c r="F66" s="19" t="n"/>
+      <c r="G66" s="20" t="n"/>
       <c r="I66" s="6" t="n">
         <v>-5685</v>
       </c>
-      <c r="J66" s="6" t="n"/>
-      <c r="K66" s="6" t="n"/>
+      <c r="J66" s="19" t="n"/>
+      <c r="K66" s="20" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="n"/>
-      <c r="B67" s="6" t="n"/>
-      <c r="C67" s="6" t="n"/>
-      <c r="E67" s="6" t="n"/>
-      <c r="F67" s="6" t="n"/>
-      <c r="G67" s="6" t="n"/>
-      <c r="I67" s="6" t="n"/>
-      <c r="J67" s="6" t="n"/>
-      <c r="K67" s="6" t="n"/>
+      <c r="A67" s="21" t="n"/>
+      <c r="B67" s="22" t="n"/>
+      <c r="C67" s="23" t="n"/>
+      <c r="E67" s="21" t="n"/>
+      <c r="F67" s="22" t="n"/>
+      <c r="G67" s="23" t="n"/>
+      <c r="I67" s="21" t="n"/>
+      <c r="J67" s="22" t="n"/>
+      <c r="K67" s="23" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -1442,84 +1553,85 @@
           <t>TWSE BFI82U 三大法人摘要，億元</t>
         </is>
       </c>
-      <c r="B68" s="7" t="n"/>
-      <c r="C68" s="7" t="n"/>
+      <c r="B68" s="19" t="n"/>
+      <c r="C68" s="20" t="n"/>
       <c r="E68" s="7" t="inlineStr">
         <is>
           <t>TWSE BFI82U 三大法人摘要，億元</t>
         </is>
       </c>
-      <c r="F68" s="7" t="n"/>
-      <c r="G68" s="7" t="n"/>
+      <c r="F68" s="19" t="n"/>
+      <c r="G68" s="20" t="n"/>
       <c r="I68" s="7" t="inlineStr">
         <is>
           <t>TAIFEX 合併口徑 = -4,400 + -5,281/4 + 710/20，四捨五入</t>
         </is>
       </c>
-      <c r="J68" s="7" t="n"/>
-      <c r="K68" s="7" t="n"/>
+      <c r="J68" s="19" t="n"/>
+      <c r="K68" s="20" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="7" t="n"/>
-      <c r="B69" s="7" t="n"/>
-      <c r="C69" s="7" t="n"/>
-      <c r="E69" s="7" t="n"/>
-      <c r="F69" s="7" t="n"/>
-      <c r="G69" s="7" t="n"/>
-      <c r="I69" s="7" t="n"/>
-      <c r="J69" s="7" t="n"/>
-      <c r="K69" s="7" t="n"/>
-    </row>
+      <c r="A69" s="21" t="n"/>
+      <c r="B69" s="22" t="n"/>
+      <c r="C69" s="23" t="n"/>
+      <c r="E69" s="21" t="n"/>
+      <c r="F69" s="22" t="n"/>
+      <c r="G69" s="23" t="n"/>
+      <c r="I69" s="21" t="n"/>
+      <c r="J69" s="22" t="n"/>
+      <c r="K69" s="23" t="n"/>
+    </row>
+    <row r="70"/>
     <row r="71">
       <c r="A71" s="13" t="inlineStr">
         <is>
           <t>自營(買)OP未平倉口數</t>
         </is>
       </c>
-      <c r="B71" s="13" t="n"/>
-      <c r="C71" s="13" t="n"/>
+      <c r="B71" s="17" t="n"/>
+      <c r="C71" s="18" t="n"/>
       <c r="E71" s="13" t="inlineStr">
         <is>
           <t>自營(買)OP未平倉金額</t>
         </is>
       </c>
-      <c r="F71" s="13" t="n"/>
-      <c r="G71" s="13" t="n"/>
+      <c r="F71" s="17" t="n"/>
+      <c r="G71" s="18" t="n"/>
       <c r="I71" s="13" t="inlineStr">
         <is>
           <t>自營(BC)OP未平倉金額與結算比</t>
         </is>
       </c>
-      <c r="J71" s="13" t="n"/>
-      <c r="K71" s="13" t="n"/>
+      <c r="J71" s="17" t="n"/>
+      <c r="K71" s="18" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="n">
         <v>4356</v>
       </c>
-      <c r="B72" s="6" t="n"/>
-      <c r="C72" s="6" t="n"/>
+      <c r="B72" s="19" t="n"/>
+      <c r="C72" s="20" t="n"/>
       <c r="E72" s="6" t="n">
         <v>-46891</v>
       </c>
-      <c r="F72" s="6" t="n"/>
-      <c r="G72" s="6" t="n"/>
+      <c r="F72" s="19" t="n"/>
+      <c r="G72" s="20" t="n"/>
       <c r="I72" s="6" t="n">
         <v>256082</v>
       </c>
-      <c r="J72" s="6" t="n"/>
-      <c r="K72" s="6" t="n"/>
+      <c r="J72" s="19" t="n"/>
+      <c r="K72" s="20" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="n"/>
-      <c r="B73" s="6" t="n"/>
-      <c r="C73" s="6" t="n"/>
-      <c r="E73" s="6" t="n"/>
-      <c r="F73" s="6" t="n"/>
-      <c r="G73" s="6" t="n"/>
-      <c r="I73" s="6" t="n"/>
-      <c r="J73" s="6" t="n"/>
-      <c r="K73" s="6" t="n"/>
+      <c r="A73" s="21" t="n"/>
+      <c r="B73" s="22" t="n"/>
+      <c r="C73" s="23" t="n"/>
+      <c r="E73" s="21" t="n"/>
+      <c r="F73" s="22" t="n"/>
+      <c r="G73" s="23" t="n"/>
+      <c r="I73" s="21" t="n"/>
+      <c r="J73" s="22" t="n"/>
+      <c r="K73" s="23" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -1527,84 +1639,85 @@
           <t>BC - SC / TAIFEX 選擇權買賣權分計</t>
         </is>
       </c>
-      <c r="B74" s="7" t="n"/>
-      <c r="C74" s="7" t="n"/>
+      <c r="B74" s="19" t="n"/>
+      <c r="C74" s="20" t="n"/>
       <c r="E74" s="7" t="inlineStr">
         <is>
           <t>BC金額 - SC金額，仟元</t>
         </is>
       </c>
-      <c r="F74" s="7" t="n"/>
-      <c r="G74" s="7" t="n"/>
+      <c r="F74" s="19" t="n"/>
+      <c r="G74" s="20" t="n"/>
       <c r="I74" s="7" t="inlineStr">
         <is>
           <t>1,427,244 - 1,171,162(4/15結算日 BC 原始金額)</t>
         </is>
       </c>
-      <c r="J74" s="7" t="n"/>
-      <c r="K74" s="7" t="n"/>
+      <c r="J74" s="19" t="n"/>
+      <c r="K74" s="20" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="7" t="n"/>
-      <c r="B75" s="7" t="n"/>
-      <c r="C75" s="7" t="n"/>
-      <c r="E75" s="7" t="n"/>
-      <c r="F75" s="7" t="n"/>
-      <c r="G75" s="7" t="n"/>
-      <c r="I75" s="7" t="n"/>
-      <c r="J75" s="7" t="n"/>
-      <c r="K75" s="7" t="n"/>
-    </row>
+      <c r="A75" s="21" t="n"/>
+      <c r="B75" s="22" t="n"/>
+      <c r="C75" s="23" t="n"/>
+      <c r="E75" s="21" t="n"/>
+      <c r="F75" s="22" t="n"/>
+      <c r="G75" s="23" t="n"/>
+      <c r="I75" s="21" t="n"/>
+      <c r="J75" s="22" t="n"/>
+      <c r="K75" s="23" t="n"/>
+    </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="13" t="inlineStr">
         <is>
           <t>自營(賣)OP未平倉口數</t>
         </is>
       </c>
-      <c r="B77" s="13" t="n"/>
-      <c r="C77" s="13" t="n"/>
+      <c r="B77" s="17" t="n"/>
+      <c r="C77" s="18" t="n"/>
       <c r="E77" s="13" t="inlineStr">
         <is>
           <t>自營(賣)OP未平倉金額</t>
         </is>
       </c>
-      <c r="F77" s="13" t="n"/>
-      <c r="G77" s="13" t="n"/>
+      <c r="F77" s="17" t="n"/>
+      <c r="G77" s="18" t="n"/>
       <c r="I77" s="13" t="inlineStr">
         <is>
           <t>自營(BP)OP未平倉金額與結算比</t>
         </is>
       </c>
-      <c r="J77" s="13" t="n"/>
-      <c r="K77" s="13" t="n"/>
+      <c r="J77" s="17" t="n"/>
+      <c r="K77" s="18" t="n"/>
     </row>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="6" t="n">
         <v>6628</v>
       </c>
-      <c r="B78" s="6" t="n"/>
-      <c r="C78" s="6" t="n"/>
+      <c r="B78" s="19" t="n"/>
+      <c r="C78" s="20" t="n"/>
       <c r="E78" s="6" t="n">
         <v>33877</v>
       </c>
-      <c r="F78" s="6" t="n"/>
-      <c r="G78" s="6" t="n"/>
+      <c r="F78" s="19" t="n"/>
+      <c r="G78" s="20" t="n"/>
       <c r="I78" s="6" t="n">
         <v>-23505</v>
       </c>
-      <c r="J78" s="6" t="n"/>
-      <c r="K78" s="6" t="n"/>
+      <c r="J78" s="19" t="n"/>
+      <c r="K78" s="20" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="6" t="n"/>
-      <c r="B79" s="6" t="n"/>
-      <c r="C79" s="6" t="n"/>
-      <c r="E79" s="6" t="n"/>
-      <c r="F79" s="6" t="n"/>
-      <c r="G79" s="6" t="n"/>
-      <c r="I79" s="6" t="n"/>
-      <c r="J79" s="6" t="n"/>
-      <c r="K79" s="6" t="n"/>
+      <c r="A79" s="21" t="n"/>
+      <c r="B79" s="22" t="n"/>
+      <c r="C79" s="23" t="n"/>
+      <c r="E79" s="21" t="n"/>
+      <c r="F79" s="22" t="n"/>
+      <c r="G79" s="23" t="n"/>
+      <c r="I79" s="21" t="n"/>
+      <c r="J79" s="22" t="n"/>
+      <c r="K79" s="23" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -1612,68 +1725,69 @@
           <t>BP - SP / TAIFEX 選擇權買賣權分計</t>
         </is>
       </c>
-      <c r="B80" s="7" t="n"/>
-      <c r="C80" s="7" t="n"/>
+      <c r="B80" s="19" t="n"/>
+      <c r="C80" s="20" t="n"/>
       <c r="E80" s="7" t="inlineStr">
         <is>
           <t>BP金額 - SP金額，仟元</t>
         </is>
       </c>
-      <c r="F80" s="7" t="n"/>
-      <c r="G80" s="7" t="n"/>
+      <c r="F80" s="19" t="n"/>
+      <c r="G80" s="20" t="n"/>
       <c r="I80" s="7" t="inlineStr">
         <is>
           <t>242,314 - 265,819(4/15結算日 BP 原始金額)</t>
         </is>
       </c>
-      <c r="J80" s="7" t="n"/>
-      <c r="K80" s="7" t="n"/>
+      <c r="J80" s="19" t="n"/>
+      <c r="K80" s="20" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="7" t="n"/>
-      <c r="B81" s="7" t="n"/>
-      <c r="C81" s="7" t="n"/>
-      <c r="E81" s="7" t="n"/>
-      <c r="F81" s="7" t="n"/>
-      <c r="G81" s="7" t="n"/>
-      <c r="I81" s="7" t="n"/>
-      <c r="J81" s="7" t="n"/>
-      <c r="K81" s="7" t="n"/>
-    </row>
+      <c r="A81" s="21" t="n"/>
+      <c r="B81" s="22" t="n"/>
+      <c r="C81" s="23" t="n"/>
+      <c r="E81" s="21" t="n"/>
+      <c r="F81" s="22" t="n"/>
+      <c r="G81" s="23" t="n"/>
+      <c r="I81" s="21" t="n"/>
+      <c r="J81" s="22" t="n"/>
+      <c r="K81" s="23" t="n"/>
+    </row>
+    <row r="82"/>
     <row r="83">
       <c r="A83" s="13" t="inlineStr">
         <is>
           <t>自營買方買權/賣權比</t>
         </is>
       </c>
-      <c r="B83" s="13" t="n"/>
-      <c r="C83" s="13" t="n"/>
+      <c r="B83" s="17" t="n"/>
+      <c r="C83" s="18" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="6" t="n">
-        <v>0.8240207833733013</v>
-      </c>
-      <c r="B84" s="6" t="n"/>
-      <c r="C84" s="6" t="n"/>
+        <v>5.890060004787177</v>
+      </c>
+      <c r="B84" s="19" t="n"/>
+      <c r="C84" s="20" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="6" t="n"/>
-      <c r="B85" s="6" t="n"/>
-      <c r="C85" s="6" t="n"/>
+      <c r="A85" s="21" t="n"/>
+      <c r="B85" s="22" t="n"/>
+      <c r="C85" s="23" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>20,617 / 25,020</t>
-        </is>
-      </c>
-      <c r="B86" s="7" t="n"/>
-      <c r="C86" s="7" t="n"/>
+          <t>1,427,244 / 242,314</t>
+        </is>
+      </c>
+      <c r="B86" s="19" t="n"/>
+      <c r="C86" s="20" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="7" t="n"/>
-      <c r="B87" s="7" t="n"/>
-      <c r="C87" s="7" t="n"/>
+      <c r="A87" s="21" t="n"/>
+      <c r="B87" s="22" t="n"/>
+      <c r="C87" s="23" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
@@ -1681,19 +1795,19 @@
           <t>散戶</t>
         </is>
       </c>
-      <c r="B90" s="4" t="n"/>
-      <c r="C90" s="4" t="n"/>
-      <c r="D90" s="4" t="n"/>
-      <c r="E90" s="4" t="n"/>
-      <c r="F90" s="4" t="n"/>
-      <c r="G90" s="4" t="n"/>
-      <c r="H90" s="4" t="n"/>
-      <c r="I90" s="4" t="n"/>
-      <c r="J90" s="4" t="n"/>
-      <c r="K90" s="4" t="n"/>
-      <c r="L90" s="4" t="n"/>
-      <c r="M90" s="4" t="n"/>
-      <c r="N90" s="4" t="n"/>
+      <c r="B90" s="17" t="n"/>
+      <c r="C90" s="17" t="n"/>
+      <c r="D90" s="17" t="n"/>
+      <c r="E90" s="17" t="n"/>
+      <c r="F90" s="17" t="n"/>
+      <c r="G90" s="17" t="n"/>
+      <c r="H90" s="17" t="n"/>
+      <c r="I90" s="17" t="n"/>
+      <c r="J90" s="17" t="n"/>
+      <c r="K90" s="17" t="n"/>
+      <c r="L90" s="17" t="n"/>
+      <c r="M90" s="17" t="n"/>
+      <c r="N90" s="18" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="15" t="inlineStr">
@@ -1701,50 +1815,50 @@
           <t>散戶看多</t>
         </is>
       </c>
-      <c r="B91" s="15" t="n"/>
-      <c r="C91" s="15" t="n"/>
+      <c r="B91" s="17" t="n"/>
+      <c r="C91" s="18" t="n"/>
       <c r="E91" s="15" t="inlineStr">
         <is>
           <t>散戶看空</t>
         </is>
       </c>
-      <c r="F91" s="15" t="n"/>
-      <c r="G91" s="15" t="n"/>
+      <c r="F91" s="17" t="n"/>
+      <c r="G91" s="18" t="n"/>
       <c r="I91" s="15" t="inlineStr">
         <is>
           <t>當次月小台留倉差增減</t>
         </is>
       </c>
-      <c r="J91" s="15" t="n"/>
-      <c r="K91" s="15" t="n"/>
+      <c r="J91" s="17" t="n"/>
+      <c r="K91" s="18" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="6" t="n">
         <v>29001</v>
       </c>
-      <c r="B92" s="6" t="n"/>
-      <c r="C92" s="6" t="n"/>
+      <c r="B92" s="19" t="n"/>
+      <c r="C92" s="20" t="n"/>
       <c r="E92" s="6" t="n">
         <v>25131</v>
       </c>
-      <c r="F92" s="6" t="n"/>
-      <c r="G92" s="6" t="n"/>
+      <c r="F92" s="19" t="n"/>
+      <c r="G92" s="20" t="n"/>
       <c r="I92" s="6" t="n">
         <v>-404</v>
       </c>
-      <c r="J92" s="6" t="n"/>
-      <c r="K92" s="6" t="n"/>
+      <c r="J92" s="19" t="n"/>
+      <c r="K92" s="20" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="6" t="n"/>
-      <c r="B93" s="6" t="n"/>
-      <c r="C93" s="6" t="n"/>
-      <c r="E93" s="6" t="n"/>
-      <c r="F93" s="6" t="n"/>
-      <c r="G93" s="6" t="n"/>
-      <c r="I93" s="6" t="n"/>
-      <c r="J93" s="6" t="n"/>
-      <c r="K93" s="6" t="n"/>
+      <c r="A93" s="21" t="n"/>
+      <c r="B93" s="22" t="n"/>
+      <c r="C93" s="23" t="n"/>
+      <c r="E93" s="21" t="n"/>
+      <c r="F93" s="22" t="n"/>
+      <c r="G93" s="23" t="n"/>
+      <c r="I93" s="21" t="n"/>
+      <c r="J93" s="22" t="n"/>
+      <c r="K93" s="23" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -1752,33 +1866,33 @@
           <t>MTX 全市場OI 36,587 - (自營3,627 + 投信116 + 外資3,843)</t>
         </is>
       </c>
-      <c r="B94" s="7" t="n"/>
-      <c r="C94" s="7" t="n"/>
+      <c r="B94" s="19" t="n"/>
+      <c r="C94" s="20" t="n"/>
       <c r="E94" s="7" t="inlineStr">
         <is>
           <t>MTX 全市場OI 36,587 - (自營8,908 + 投信39 + 外資2,509)</t>
         </is>
       </c>
-      <c r="F94" s="7" t="n"/>
-      <c r="G94" s="7" t="n"/>
+      <c r="F94" s="19" t="n"/>
+      <c r="G94" s="20" t="n"/>
       <c r="I94" s="7" t="inlineStr">
         <is>
           <t>(29,090-4,175) - (29,261-3,942)</t>
         </is>
       </c>
-      <c r="J94" s="7" t="n"/>
-      <c r="K94" s="7" t="n"/>
+      <c r="J94" s="19" t="n"/>
+      <c r="K94" s="20" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="7" t="n"/>
-      <c r="B95" s="7" t="n"/>
-      <c r="C95" s="7" t="n"/>
-      <c r="E95" s="7" t="n"/>
-      <c r="F95" s="7" t="n"/>
-      <c r="G95" s="7" t="n"/>
-      <c r="I95" s="7" t="n"/>
-      <c r="J95" s="7" t="n"/>
-      <c r="K95" s="7" t="n"/>
+      <c r="A95" s="21" t="n"/>
+      <c r="B95" s="22" t="n"/>
+      <c r="C95" s="23" t="n"/>
+      <c r="E95" s="21" t="n"/>
+      <c r="F95" s="22" t="n"/>
+      <c r="G95" s="23" t="n"/>
+      <c r="I95" s="21" t="n"/>
+      <c r="J95" s="22" t="n"/>
+      <c r="K95" s="23" t="n"/>
     </row>
     <row r="96" ht="32" customHeight="1"/>
     <row r="97">
@@ -1787,50 +1901,50 @@
           <t>散戶未平倉</t>
         </is>
       </c>
-      <c r="B97" s="15" t="n"/>
-      <c r="C97" s="15" t="n"/>
+      <c r="B97" s="17" t="n"/>
+      <c r="C97" s="18" t="n"/>
       <c r="E97" s="15" t="inlineStr">
         <is>
           <t>微台散戶看多</t>
         </is>
       </c>
-      <c r="F97" s="15" t="n"/>
-      <c r="G97" s="15" t="n"/>
+      <c r="F97" s="17" t="n"/>
+      <c r="G97" s="18" t="n"/>
       <c r="I97" s="15" t="inlineStr">
         <is>
           <t>微台散戶看空</t>
         </is>
       </c>
-      <c r="J97" s="15" t="n"/>
-      <c r="K97" s="15" t="n"/>
+      <c r="J97" s="17" t="n"/>
+      <c r="K97" s="18" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="6" t="n">
         <v>3870</v>
       </c>
-      <c r="B98" s="6" t="n"/>
-      <c r="C98" s="6" t="n"/>
+      <c r="B98" s="19" t="n"/>
+      <c r="C98" s="20" t="n"/>
       <c r="E98" s="6" t="n">
         <v>42282</v>
       </c>
-      <c r="F98" s="6" t="n"/>
-      <c r="G98" s="6" t="n"/>
+      <c r="F98" s="19" t="n"/>
+      <c r="G98" s="20" t="n"/>
       <c r="I98" s="6" t="n">
         <v>45118</v>
       </c>
-      <c r="J98" s="6" t="n"/>
-      <c r="K98" s="6" t="n"/>
+      <c r="J98" s="19" t="n"/>
+      <c r="K98" s="20" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="6" t="n"/>
-      <c r="B99" s="6" t="n"/>
-      <c r="C99" s="6" t="n"/>
-      <c r="E99" s="6" t="n"/>
-      <c r="F99" s="6" t="n"/>
-      <c r="G99" s="6" t="n"/>
-      <c r="I99" s="6" t="n"/>
-      <c r="J99" s="6" t="n"/>
-      <c r="K99" s="6" t="n"/>
+      <c r="A99" s="21" t="n"/>
+      <c r="B99" s="22" t="n"/>
+      <c r="C99" s="23" t="n"/>
+      <c r="E99" s="21" t="n"/>
+      <c r="F99" s="22" t="n"/>
+      <c r="G99" s="23" t="n"/>
+      <c r="I99" s="21" t="n"/>
+      <c r="J99" s="22" t="n"/>
+      <c r="K99" s="23" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -1838,33 +1952,33 @@
           <t>29,001 - 25,131</t>
         </is>
       </c>
-      <c r="B100" s="7" t="n"/>
-      <c r="C100" s="7" t="n"/>
+      <c r="B100" s="19" t="n"/>
+      <c r="C100" s="20" t="n"/>
       <c r="E100" s="7" t="inlineStr">
         <is>
           <t>TMF 全市場OI 49,851 - (自營5,034 + 投信0 + 外資2,535)</t>
         </is>
       </c>
-      <c r="F100" s="7" t="n"/>
-      <c r="G100" s="7" t="n"/>
+      <c r="F100" s="19" t="n"/>
+      <c r="G100" s="20" t="n"/>
       <c r="I100" s="7" t="inlineStr">
         <is>
           <t>TMF 全市場OI 49,851 - (自營4,324 + 投信0 + 外資409)</t>
         </is>
       </c>
-      <c r="J100" s="7" t="n"/>
-      <c r="K100" s="7" t="n"/>
+      <c r="J100" s="19" t="n"/>
+      <c r="K100" s="20" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="7" t="n"/>
-      <c r="B101" s="7" t="n"/>
-      <c r="C101" s="7" t="n"/>
-      <c r="E101" s="7" t="n"/>
-      <c r="F101" s="7" t="n"/>
-      <c r="G101" s="7" t="n"/>
-      <c r="I101" s="7" t="n"/>
-      <c r="J101" s="7" t="n"/>
-      <c r="K101" s="7" t="n"/>
+      <c r="A101" s="21" t="n"/>
+      <c r="B101" s="22" t="n"/>
+      <c r="C101" s="23" t="n"/>
+      <c r="E101" s="21" t="n"/>
+      <c r="F101" s="22" t="n"/>
+      <c r="G101" s="23" t="n"/>
+      <c r="I101" s="21" t="n"/>
+      <c r="J101" s="22" t="n"/>
+      <c r="K101" s="23" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="15" t="inlineStr">
@@ -1872,35 +1986,35 @@
           <t>微台散戶多空比</t>
         </is>
       </c>
-      <c r="B103" s="15" t="n"/>
-      <c r="C103" s="15" t="n"/>
+      <c r="B103" s="17" t="n"/>
+      <c r="C103" s="18" t="n"/>
       <c r="E103" s="15" t="inlineStr">
         <is>
           <t>微台散戶未平倉</t>
         </is>
       </c>
-      <c r="F103" s="15" t="n"/>
-      <c r="G103" s="15" t="n"/>
+      <c r="F103" s="17" t="n"/>
+      <c r="G103" s="18" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="6" t="n">
         <v>-5.688953080178933</v>
       </c>
-      <c r="B104" s="6" t="n"/>
-      <c r="C104" s="6" t="n"/>
+      <c r="B104" s="19" t="n"/>
+      <c r="C104" s="20" t="n"/>
       <c r="E104" s="6" t="n">
         <v>-2836</v>
       </c>
-      <c r="F104" s="6" t="n"/>
-      <c r="G104" s="6" t="n"/>
+      <c r="F104" s="19" t="n"/>
+      <c r="G104" s="20" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="6" t="n"/>
-      <c r="B105" s="6" t="n"/>
-      <c r="C105" s="6" t="n"/>
-      <c r="E105" s="6" t="n"/>
-      <c r="F105" s="6" t="n"/>
-      <c r="G105" s="6" t="n"/>
+      <c r="A105" s="21" t="n"/>
+      <c r="B105" s="22" t="n"/>
+      <c r="C105" s="23" t="n"/>
+      <c r="E105" s="21" t="n"/>
+      <c r="F105" s="22" t="n"/>
+      <c r="G105" s="23" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -1908,23 +2022,23 @@
           <t>(-2,836 / 49,851) x 100</t>
         </is>
       </c>
-      <c r="B106" s="7" t="n"/>
-      <c r="C106" s="7" t="n"/>
+      <c r="B106" s="19" t="n"/>
+      <c r="C106" s="20" t="n"/>
       <c r="E106" s="7" t="inlineStr">
         <is>
           <t>42,282 - 45,118</t>
         </is>
       </c>
-      <c r="F106" s="7" t="n"/>
-      <c r="G106" s="7" t="n"/>
+      <c r="F106" s="19" t="n"/>
+      <c r="G106" s="20" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="7" t="n"/>
-      <c r="B107" s="7" t="n"/>
-      <c r="C107" s="7" t="n"/>
-      <c r="E107" s="7" t="n"/>
-      <c r="F107" s="7" t="n"/>
-      <c r="G107" s="7" t="n"/>
+      <c r="A107" s="21" t="n"/>
+      <c r="B107" s="22" t="n"/>
+      <c r="C107" s="23" t="n"/>
+      <c r="E107" s="21" t="n"/>
+      <c r="F107" s="22" t="n"/>
+      <c r="G107" s="23" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
@@ -2126,19 +2240,19 @@
           <t>大盤概況</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
+      <c r="B4" s="17" t="n"/>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="17" t="n"/>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="17" t="n"/>
+      <c r="M4" s="17" t="n"/>
+      <c r="N4" s="18" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -2146,22 +2260,22 @@
           <t>日期</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n"/>
-      <c r="C5" s="9" t="n"/>
+      <c r="B5" s="17" t="n"/>
+      <c r="C5" s="18" t="n"/>
       <c r="E5" s="9" t="inlineStr">
         <is>
           <t>結算日</t>
         </is>
       </c>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="18" t="n"/>
       <c r="I5" s="9" t="inlineStr">
         <is>
           <t>當次月大台留倉差增減</t>
         </is>
       </c>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2169,29 +2283,29 @@
           <t>2026-04-22</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="20" t="n"/>
       <c r="E6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="20" t="n"/>
       <c r="I6" s="6" t="n">
         <v>-926</v>
       </c>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
+      <c r="J6" s="19" t="n"/>
+      <c r="K6" s="20" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="6" t="n"/>
+      <c r="A7" s="21" t="n"/>
+      <c r="B7" s="22" t="n"/>
+      <c r="C7" s="23" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="23" t="n"/>
+      <c r="I7" s="21" t="n"/>
+      <c r="J7" s="22" t="n"/>
+      <c r="K7" s="23" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2199,33 +2313,33 @@
           <t>今日日盤後整理</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="20" t="n"/>
       <c r="E8" s="7" t="inlineStr">
         <is>
           <t>原表編碼對應星期三</t>
         </is>
       </c>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="20" t="n"/>
       <c r="I8" s="7" t="inlineStr">
         <is>
           <t>(81,421-2,122) - (82,127-1,902)</t>
         </is>
       </c>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="20" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
+      <c r="A9" s="21" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="23" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="23" t="n"/>
+      <c r="I9" s="21" t="n"/>
+      <c r="J9" s="22" t="n"/>
+      <c r="K9" s="23" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2233,50 +2347,50 @@
           <t>加權指數</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
+      <c r="B11" s="17" t="n"/>
+      <c r="C11" s="18" t="n"/>
       <c r="E11" s="9" t="inlineStr">
         <is>
           <t>加權指數漲跌</t>
         </is>
       </c>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
+      <c r="F11" s="17" t="n"/>
+      <c r="G11" s="18" t="n"/>
       <c r="I11" s="9" t="inlineStr">
         <is>
           <t>加權指數漲跌幅(%)</t>
         </is>
       </c>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="18" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="6" t="n">
         <v>37878.47</v>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
+      <c r="B12" s="19" t="n"/>
+      <c r="C12" s="20" t="n"/>
       <c r="E12" s="6" t="n">
         <v>273.36</v>
       </c>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="20" t="n"/>
       <c r="I12" s="6" t="n">
         <v>0.73</v>
       </c>
-      <c r="J12" s="6" t="n"/>
-      <c r="K12" s="6" t="n"/>
+      <c r="J12" s="19" t="n"/>
+      <c r="K12" s="20" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="6" t="n"/>
+      <c r="A13" s="21" t="n"/>
+      <c r="B13" s="22" t="n"/>
+      <c r="C13" s="23" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="22" t="n"/>
+      <c r="G13" s="23" t="n"/>
+      <c r="I13" s="21" t="n"/>
+      <c r="J13" s="22" t="n"/>
+      <c r="K13" s="23" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -2284,33 +2398,33 @@
           <t>TWSE MI_INDEX</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="20" t="n"/>
       <c r="E14" s="7" t="inlineStr">
         <is>
           <t>TWSE MI_INDEX</t>
         </is>
       </c>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="20" t="n"/>
       <c r="I14" s="7" t="inlineStr">
         <is>
           <t>TWSE MI_INDEX</t>
         </is>
       </c>
-      <c r="J14" s="7" t="n"/>
-      <c r="K14" s="7" t="n"/>
+      <c r="J14" s="19" t="n"/>
+      <c r="K14" s="20" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
+      <c r="A15" s="21" t="n"/>
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="23" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="22" t="n"/>
+      <c r="G15" s="23" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="22" t="n"/>
+      <c r="K15" s="23" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
@@ -2318,19 +2432,19 @@
           <t>外資選擇權細項</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="n"/>
-      <c r="L18" s="4" t="n"/>
-      <c r="M18" s="4" t="n"/>
-      <c r="N18" s="4" t="n"/>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="17" t="n"/>
+      <c r="H18" s="17" t="n"/>
+      <c r="I18" s="17" t="n"/>
+      <c r="J18" s="17" t="n"/>
+      <c r="K18" s="17" t="n"/>
+      <c r="L18" s="17" t="n"/>
+      <c r="M18" s="17" t="n"/>
+      <c r="N18" s="18" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -2338,50 +2452,50 @@
           <t>外資BC口數</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="18" t="n"/>
       <c r="E19" s="11" t="inlineStr">
         <is>
           <t>外資BC金額</t>
         </is>
       </c>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="18" t="n"/>
       <c r="I19" s="11" t="inlineStr">
         <is>
           <t>外資SC口數</t>
         </is>
       </c>
-      <c r="J19" s="11" t="n"/>
-      <c r="K19" s="11" t="n"/>
+      <c r="J19" s="17" t="n"/>
+      <c r="K19" s="18" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
         <v>7510</v>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="20" t="n"/>
       <c r="E20" s="6" t="n">
         <v>1098547</v>
       </c>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="20" t="n"/>
       <c r="I20" s="6" t="n">
         <v>7858</v>
       </c>
-      <c r="J20" s="6" t="n"/>
-      <c r="K20" s="6" t="n"/>
+      <c r="J20" s="19" t="n"/>
+      <c r="K20" s="20" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="I21" s="6" t="n"/>
-      <c r="J21" s="6" t="n"/>
-      <c r="K21" s="6" t="n"/>
+      <c r="A21" s="21" t="n"/>
+      <c r="B21" s="22" t="n"/>
+      <c r="C21" s="23" t="n"/>
+      <c r="E21" s="21" t="n"/>
+      <c r="F21" s="22" t="n"/>
+      <c r="G21" s="23" t="n"/>
+      <c r="I21" s="21" t="n"/>
+      <c r="J21" s="22" t="n"/>
+      <c r="K21" s="23" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2389,33 +2503,33 @@
           <t>買權買方</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="20" t="n"/>
       <c r="E22" s="7" t="inlineStr">
         <is>
           <t>仟元</t>
         </is>
       </c>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="20" t="n"/>
       <c r="I22" s="7" t="inlineStr">
         <is>
           <t>買權賣方</t>
         </is>
       </c>
-      <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
+      <c r="J22" s="19" t="n"/>
+      <c r="K22" s="20" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="n"/>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="22" t="n"/>
+      <c r="C23" s="23" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="22" t="n"/>
+      <c r="G23" s="23" t="n"/>
+      <c r="I23" s="21" t="n"/>
+      <c r="J23" s="22" t="n"/>
+      <c r="K23" s="23" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -2423,50 +2537,50 @@
           <t>外資SC金額</t>
         </is>
       </c>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="18" t="n"/>
       <c r="E25" s="11" t="inlineStr">
         <is>
           <t>外資(SC增幅-BC增幅)金額</t>
         </is>
       </c>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
+      <c r="F25" s="17" t="n"/>
+      <c r="G25" s="18" t="n"/>
       <c r="I25" s="11" t="inlineStr">
         <is>
           <t>外資BC/SC增幅比例</t>
         </is>
       </c>
-      <c r="J25" s="11" t="n"/>
-      <c r="K25" s="11" t="n"/>
+      <c r="J25" s="17" t="n"/>
+      <c r="K25" s="18" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
         <v>902853</v>
       </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="20" t="n"/>
       <c r="E26" s="6" t="n">
         <v>6189</v>
       </c>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="20" t="n"/>
       <c r="I26" s="6" t="n">
         <v>0.3719298245614035</v>
       </c>
-      <c r="J26" s="6" t="n"/>
-      <c r="K26" s="6" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="20" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="J27" s="6" t="n"/>
-      <c r="K27" s="6" t="n"/>
+      <c r="A27" s="21" t="n"/>
+      <c r="B27" s="22" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="22" t="n"/>
+      <c r="G27" s="23" t="n"/>
+      <c r="I27" s="21" t="n"/>
+      <c r="J27" s="22" t="n"/>
+      <c r="K27" s="23" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2474,33 +2588,33 @@
           <t>仟元</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="n"/>
+      <c r="B28" s="19" t="n"/>
+      <c r="C28" s="20" t="n"/>
       <c r="E28" s="7" t="inlineStr">
         <is>
           <t>(902,853-903,024) - (1,098,547-1,104,907)</t>
         </is>
       </c>
-      <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="20" t="n"/>
       <c r="I28" s="7" t="inlineStr">
         <is>
           <t>(1,098,547-1,104,907) / (902,853-903,024) / 100</t>
         </is>
       </c>
-      <c r="J28" s="7" t="n"/>
-      <c r="K28" s="7" t="n"/>
+      <c r="J28" s="19" t="n"/>
+      <c r="K28" s="20" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
-      <c r="F29" s="7" t="n"/>
-      <c r="G29" s="7" t="n"/>
-      <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="n"/>
+      <c r="A29" s="21" t="n"/>
+      <c r="B29" s="22" t="n"/>
+      <c r="C29" s="23" t="n"/>
+      <c r="E29" s="21" t="n"/>
+      <c r="F29" s="22" t="n"/>
+      <c r="G29" s="23" t="n"/>
+      <c r="I29" s="21" t="n"/>
+      <c r="J29" s="22" t="n"/>
+      <c r="K29" s="23" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -2508,50 +2622,50 @@
           <t>外資BP口數</t>
         </is>
       </c>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="11" t="n"/>
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="18" t="n"/>
       <c r="E31" s="11" t="inlineStr">
         <is>
           <t>外資BP金額</t>
         </is>
       </c>
-      <c r="F31" s="11" t="n"/>
-      <c r="G31" s="11" t="n"/>
+      <c r="F31" s="17" t="n"/>
+      <c r="G31" s="18" t="n"/>
       <c r="I31" s="11" t="inlineStr">
         <is>
           <t>外資SP口數</t>
         </is>
       </c>
-      <c r="J31" s="11" t="n"/>
-      <c r="K31" s="11" t="n"/>
+      <c r="J31" s="17" t="n"/>
+      <c r="K31" s="18" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="6" t="n">
         <v>11363</v>
       </c>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="6" t="n"/>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="20" t="n"/>
       <c r="E32" s="6" t="n">
         <v>125723</v>
       </c>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="20" t="n"/>
       <c r="I32" s="6" t="n">
         <v>11362</v>
       </c>
-      <c r="J32" s="6" t="n"/>
-      <c r="K32" s="6" t="n"/>
+      <c r="J32" s="19" t="n"/>
+      <c r="K32" s="20" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="6" t="n"/>
-      <c r="I33" s="6" t="n"/>
-      <c r="J33" s="6" t="n"/>
-      <c r="K33" s="6" t="n"/>
+      <c r="A33" s="21" t="n"/>
+      <c r="B33" s="22" t="n"/>
+      <c r="C33" s="23" t="n"/>
+      <c r="E33" s="21" t="n"/>
+      <c r="F33" s="22" t="n"/>
+      <c r="G33" s="23" t="n"/>
+      <c r="I33" s="21" t="n"/>
+      <c r="J33" s="22" t="n"/>
+      <c r="K33" s="23" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2559,33 +2673,33 @@
           <t>賣權買方</t>
         </is>
       </c>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="20" t="n"/>
       <c r="E34" s="7" t="inlineStr">
         <is>
           <t>仟元</t>
         </is>
       </c>
-      <c r="F34" s="7" t="n"/>
-      <c r="G34" s="7" t="n"/>
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="20" t="n"/>
       <c r="I34" s="7" t="inlineStr">
         <is>
           <t>賣權賣方</t>
         </is>
       </c>
-      <c r="J34" s="7" t="n"/>
-      <c r="K34" s="7" t="n"/>
+      <c r="J34" s="19" t="n"/>
+      <c r="K34" s="20" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="n"/>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="n"/>
-      <c r="G35" s="7" t="n"/>
-      <c r="I35" s="7" t="n"/>
-      <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="n"/>
+      <c r="A35" s="21" t="n"/>
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="23" t="n"/>
+      <c r="E35" s="21" t="n"/>
+      <c r="F35" s="22" t="n"/>
+      <c r="G35" s="23" t="n"/>
+      <c r="I35" s="21" t="n"/>
+      <c r="J35" s="22" t="n"/>
+      <c r="K35" s="23" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -2593,50 +2707,50 @@
           <t>外資SP金額</t>
         </is>
       </c>
-      <c r="B37" s="11" t="n"/>
-      <c r="C37" s="11" t="n"/>
+      <c r="B37" s="17" t="n"/>
+      <c r="C37" s="18" t="n"/>
       <c r="E37" s="11" t="inlineStr">
         <is>
           <t>外資(SP增幅-BP增幅)金額</t>
         </is>
       </c>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
+      <c r="F37" s="17" t="n"/>
+      <c r="G37" s="18" t="n"/>
       <c r="I37" s="11" t="inlineStr">
         <is>
           <t>外資BP/SP增幅比例</t>
         </is>
       </c>
-      <c r="J37" s="11" t="n"/>
-      <c r="K37" s="11" t="n"/>
+      <c r="J37" s="17" t="n"/>
+      <c r="K37" s="18" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
         <v>108859</v>
       </c>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="20" t="n"/>
       <c r="E38" s="6" t="n">
         <v>-12403</v>
       </c>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
+      <c r="F38" s="19" t="n"/>
+      <c r="G38" s="20" t="n"/>
       <c r="I38" s="6" t="n">
         <v>0.003620512292973974</v>
       </c>
-      <c r="J38" s="6" t="n"/>
-      <c r="K38" s="6" t="n"/>
+      <c r="J38" s="19" t="n"/>
+      <c r="K38" s="20" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="6" t="n"/>
-      <c r="I39" s="6" t="n"/>
-      <c r="J39" s="6" t="n"/>
-      <c r="K39" s="6" t="n"/>
+      <c r="A39" s="21" t="n"/>
+      <c r="B39" s="22" t="n"/>
+      <c r="C39" s="23" t="n"/>
+      <c r="E39" s="21" t="n"/>
+      <c r="F39" s="22" t="n"/>
+      <c r="G39" s="23" t="n"/>
+      <c r="I39" s="21" t="n"/>
+      <c r="J39" s="22" t="n"/>
+      <c r="K39" s="23" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2644,33 +2758,33 @@
           <t>仟元</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="7" t="n"/>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="20" t="n"/>
       <c r="E40" s="7" t="inlineStr">
         <is>
           <t>(108,859-128,301) - (125,723-132,762)</t>
         </is>
       </c>
-      <c r="F40" s="7" t="n"/>
-      <c r="G40" s="7" t="n"/>
+      <c r="F40" s="19" t="n"/>
+      <c r="G40" s="20" t="n"/>
       <c r="I40" s="7" t="inlineStr">
         <is>
           <t>(125,723-132,762) / (108,859-128,301) / 100</t>
         </is>
       </c>
-      <c r="J40" s="7" t="n"/>
-      <c r="K40" s="7" t="n"/>
+      <c r="J40" s="19" t="n"/>
+      <c r="K40" s="20" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="n"/>
-      <c r="B41" s="7" t="n"/>
-      <c r="C41" s="7" t="n"/>
-      <c r="E41" s="7" t="n"/>
-      <c r="F41" s="7" t="n"/>
-      <c r="G41" s="7" t="n"/>
-      <c r="I41" s="7" t="n"/>
-      <c r="J41" s="7" t="n"/>
-      <c r="K41" s="7" t="n"/>
+      <c r="A41" s="21" t="n"/>
+      <c r="B41" s="22" t="n"/>
+      <c r="C41" s="23" t="n"/>
+      <c r="E41" s="21" t="n"/>
+      <c r="F41" s="22" t="n"/>
+      <c r="G41" s="23" t="n"/>
+      <c r="I41" s="21" t="n"/>
+      <c r="J41" s="22" t="n"/>
+      <c r="K41" s="23" t="n"/>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="12" t="inlineStr">
@@ -2678,19 +2792,19 @@
           <t>自營選擇權細項</t>
         </is>
       </c>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
-      <c r="H44" s="4" t="n"/>
-      <c r="I44" s="4" t="n"/>
-      <c r="J44" s="4" t="n"/>
-      <c r="K44" s="4" t="n"/>
-      <c r="L44" s="4" t="n"/>
-      <c r="M44" s="4" t="n"/>
-      <c r="N44" s="4" t="n"/>
+      <c r="B44" s="17" t="n"/>
+      <c r="C44" s="17" t="n"/>
+      <c r="D44" s="17" t="n"/>
+      <c r="E44" s="17" t="n"/>
+      <c r="F44" s="17" t="n"/>
+      <c r="G44" s="17" t="n"/>
+      <c r="H44" s="17" t="n"/>
+      <c r="I44" s="17" t="n"/>
+      <c r="J44" s="17" t="n"/>
+      <c r="K44" s="17" t="n"/>
+      <c r="L44" s="17" t="n"/>
+      <c r="M44" s="17" t="n"/>
+      <c r="N44" s="18" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
@@ -2698,50 +2812,50 @@
           <t>自營BC口數</t>
         </is>
       </c>
-      <c r="B45" s="13" t="n"/>
-      <c r="C45" s="13" t="n"/>
+      <c r="B45" s="17" t="n"/>
+      <c r="C45" s="18" t="n"/>
       <c r="E45" s="13" t="inlineStr">
         <is>
           <t>自營BC金額</t>
         </is>
       </c>
-      <c r="F45" s="13" t="n"/>
-      <c r="G45" s="13" t="n"/>
+      <c r="F45" s="17" t="n"/>
+      <c r="G45" s="18" t="n"/>
       <c r="I45" s="13" t="inlineStr">
         <is>
           <t>自營SC口數</t>
         </is>
       </c>
-      <c r="J45" s="13" t="n"/>
-      <c r="K45" s="13" t="n"/>
+      <c r="J45" s="17" t="n"/>
+      <c r="K45" s="18" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
         <v>20617</v>
       </c>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="6" t="n"/>
+      <c r="B46" s="19" t="n"/>
+      <c r="C46" s="20" t="n"/>
       <c r="E46" s="6" t="n">
         <v>1427244</v>
       </c>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="6" t="n"/>
+      <c r="F46" s="19" t="n"/>
+      <c r="G46" s="20" t="n"/>
       <c r="I46" s="6" t="n">
         <v>16261</v>
       </c>
-      <c r="J46" s="6" t="n"/>
-      <c r="K46" s="6" t="n"/>
+      <c r="J46" s="19" t="n"/>
+      <c r="K46" s="20" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="6" t="n"/>
-      <c r="I47" s="6" t="n"/>
-      <c r="J47" s="6" t="n"/>
-      <c r="K47" s="6" t="n"/>
+      <c r="A47" s="21" t="n"/>
+      <c r="B47" s="22" t="n"/>
+      <c r="C47" s="23" t="n"/>
+      <c r="E47" s="21" t="n"/>
+      <c r="F47" s="22" t="n"/>
+      <c r="G47" s="23" t="n"/>
+      <c r="I47" s="21" t="n"/>
+      <c r="J47" s="22" t="n"/>
+      <c r="K47" s="23" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2749,33 +2863,33 @@
           <t>買權買方 / TAIFEX</t>
         </is>
       </c>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="7" t="n"/>
+      <c r="B48" s="19" t="n"/>
+      <c r="C48" s="20" t="n"/>
       <c r="E48" s="7" t="inlineStr">
         <is>
           <t>仟元</t>
         </is>
       </c>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="7" t="n"/>
+      <c r="F48" s="19" t="n"/>
+      <c r="G48" s="20" t="n"/>
       <c r="I48" s="7" t="inlineStr">
         <is>
           <t>買權賣方 / TAIFEX</t>
         </is>
       </c>
-      <c r="J48" s="7" t="n"/>
-      <c r="K48" s="7" t="n"/>
+      <c r="J48" s="19" t="n"/>
+      <c r="K48" s="20" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n"/>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="7" t="n"/>
-      <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="n"/>
-      <c r="G49" s="7" t="n"/>
-      <c r="I49" s="7" t="n"/>
-      <c r="J49" s="7" t="n"/>
-      <c r="K49" s="7" t="n"/>
+      <c r="A49" s="21" t="n"/>
+      <c r="B49" s="22" t="n"/>
+      <c r="C49" s="23" t="n"/>
+      <c r="E49" s="21" t="n"/>
+      <c r="F49" s="22" t="n"/>
+      <c r="G49" s="23" t="n"/>
+      <c r="I49" s="21" t="n"/>
+      <c r="J49" s="22" t="n"/>
+      <c r="K49" s="23" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
@@ -2783,50 +2897,50 @@
           <t>自營SC金額</t>
         </is>
       </c>
-      <c r="B51" s="13" t="n"/>
-      <c r="C51" s="13" t="n"/>
+      <c r="B51" s="17" t="n"/>
+      <c r="C51" s="18" t="n"/>
       <c r="E51" s="13" t="inlineStr">
         <is>
           <t>自營(SC增幅-BC增幅)金額</t>
         </is>
       </c>
-      <c r="F51" s="13" t="n"/>
-      <c r="G51" s="13" t="n"/>
+      <c r="F51" s="17" t="n"/>
+      <c r="G51" s="18" t="n"/>
       <c r="I51" s="13" t="inlineStr">
         <is>
           <t>自營BC/SC增幅比例</t>
         </is>
       </c>
-      <c r="J51" s="13" t="n"/>
-      <c r="K51" s="13" t="n"/>
+      <c r="J51" s="17" t="n"/>
+      <c r="K51" s="18" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
         <v>1474135</v>
       </c>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="6" t="n"/>
+      <c r="B52" s="19" t="n"/>
+      <c r="C52" s="20" t="n"/>
       <c r="E52" s="6" t="n">
         <v>-10428</v>
       </c>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="6" t="n"/>
+      <c r="F52" s="19" t="n"/>
+      <c r="G52" s="20" t="n"/>
       <c r="I52" s="6" t="n">
         <v>0.008166376536371788</v>
       </c>
-      <c r="J52" s="6" t="n"/>
-      <c r="K52" s="6" t="n"/>
+      <c r="J52" s="19" t="n"/>
+      <c r="K52" s="20" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n"/>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="6" t="n"/>
-      <c r="I53" s="6" t="n"/>
-      <c r="J53" s="6" t="n"/>
-      <c r="K53" s="6" t="n"/>
+      <c r="A53" s="21" t="n"/>
+      <c r="B53" s="22" t="n"/>
+      <c r="C53" s="23" t="n"/>
+      <c r="E53" s="21" t="n"/>
+      <c r="F53" s="22" t="n"/>
+      <c r="G53" s="23" t="n"/>
+      <c r="I53" s="21" t="n"/>
+      <c r="J53" s="22" t="n"/>
+      <c r="K53" s="23" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -2834,33 +2948,33 @@
           <t>仟元</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="7" t="n"/>
+      <c r="B54" s="19" t="n"/>
+      <c r="C54" s="20" t="n"/>
       <c r="E54" s="7" t="inlineStr">
         <is>
           <t>(1,474,135-1,531,006) - (1,427,244-1,473,687)</t>
         </is>
       </c>
-      <c r="F54" s="7" t="n"/>
-      <c r="G54" s="7" t="n"/>
+      <c r="F54" s="19" t="n"/>
+      <c r="G54" s="20" t="n"/>
       <c r="I54" s="7" t="inlineStr">
         <is>
           <t>(1,427,244-1,473,687) / (1,474,135-1,531,006) / 100</t>
         </is>
       </c>
-      <c r="J54" s="7" t="n"/>
-      <c r="K54" s="7" t="n"/>
+      <c r="J54" s="19" t="n"/>
+      <c r="K54" s="20" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="n"/>
-      <c r="B55" s="7" t="n"/>
-      <c r="C55" s="7" t="n"/>
-      <c r="E55" s="7" t="n"/>
-      <c r="F55" s="7" t="n"/>
-      <c r="G55" s="7" t="n"/>
-      <c r="I55" s="7" t="n"/>
-      <c r="J55" s="7" t="n"/>
-      <c r="K55" s="7" t="n"/>
+      <c r="A55" s="21" t="n"/>
+      <c r="B55" s="22" t="n"/>
+      <c r="C55" s="23" t="n"/>
+      <c r="E55" s="21" t="n"/>
+      <c r="F55" s="22" t="n"/>
+      <c r="G55" s="23" t="n"/>
+      <c r="I55" s="21" t="n"/>
+      <c r="J55" s="22" t="n"/>
+      <c r="K55" s="23" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="13" t="inlineStr">
@@ -2868,50 +2982,50 @@
           <t>自營BP口數</t>
         </is>
       </c>
-      <c r="B57" s="13" t="n"/>
-      <c r="C57" s="13" t="n"/>
+      <c r="B57" s="17" t="n"/>
+      <c r="C57" s="18" t="n"/>
       <c r="E57" s="13" t="inlineStr">
         <is>
           <t>自營BP金額</t>
         </is>
       </c>
-      <c r="F57" s="13" t="n"/>
-      <c r="G57" s="13" t="n"/>
+      <c r="F57" s="17" t="n"/>
+      <c r="G57" s="18" t="n"/>
       <c r="I57" s="13" t="inlineStr">
         <is>
           <t>自營SP口數</t>
         </is>
       </c>
-      <c r="J57" s="13" t="n"/>
-      <c r="K57" s="13" t="n"/>
+      <c r="J57" s="17" t="n"/>
+      <c r="K57" s="18" t="n"/>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="6" t="n">
         <v>25020</v>
       </c>
-      <c r="B58" s="6" t="n"/>
-      <c r="C58" s="6" t="n"/>
+      <c r="B58" s="19" t="n"/>
+      <c r="C58" s="20" t="n"/>
       <c r="E58" s="6" t="n">
         <v>242314</v>
       </c>
-      <c r="F58" s="6" t="n"/>
-      <c r="G58" s="6" t="n"/>
+      <c r="F58" s="19" t="n"/>
+      <c r="G58" s="20" t="n"/>
       <c r="I58" s="6" t="n">
         <v>18392</v>
       </c>
-      <c r="J58" s="6" t="n"/>
-      <c r="K58" s="6" t="n"/>
+      <c r="J58" s="19" t="n"/>
+      <c r="K58" s="20" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="n"/>
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="6" t="n"/>
-      <c r="E59" s="6" t="n"/>
-      <c r="F59" s="6" t="n"/>
-      <c r="G59" s="6" t="n"/>
-      <c r="I59" s="6" t="n"/>
-      <c r="J59" s="6" t="n"/>
-      <c r="K59" s="6" t="n"/>
+      <c r="A59" s="21" t="n"/>
+      <c r="B59" s="22" t="n"/>
+      <c r="C59" s="23" t="n"/>
+      <c r="E59" s="21" t="n"/>
+      <c r="F59" s="22" t="n"/>
+      <c r="G59" s="23" t="n"/>
+      <c r="I59" s="21" t="n"/>
+      <c r="J59" s="22" t="n"/>
+      <c r="K59" s="23" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -2919,33 +3033,33 @@
           <t>賣權買方 / TAIFEX</t>
         </is>
       </c>
-      <c r="B60" s="7" t="n"/>
-      <c r="C60" s="7" t="n"/>
+      <c r="B60" s="19" t="n"/>
+      <c r="C60" s="20" t="n"/>
       <c r="E60" s="7" t="inlineStr">
         <is>
           <t>仟元</t>
         </is>
       </c>
-      <c r="F60" s="7" t="n"/>
-      <c r="G60" s="7" t="n"/>
+      <c r="F60" s="19" t="n"/>
+      <c r="G60" s="20" t="n"/>
       <c r="I60" s="7" t="inlineStr">
         <is>
           <t>賣權賣方 / TAIFEX</t>
         </is>
       </c>
-      <c r="J60" s="7" t="n"/>
-      <c r="K60" s="7" t="n"/>
+      <c r="J60" s="19" t="n"/>
+      <c r="K60" s="20" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="n"/>
-      <c r="B61" s="7" t="n"/>
-      <c r="C61" s="7" t="n"/>
-      <c r="E61" s="7" t="n"/>
-      <c r="F61" s="7" t="n"/>
-      <c r="G61" s="7" t="n"/>
-      <c r="I61" s="7" t="n"/>
-      <c r="J61" s="7" t="n"/>
-      <c r="K61" s="7" t="n"/>
+      <c r="A61" s="21" t="n"/>
+      <c r="B61" s="22" t="n"/>
+      <c r="C61" s="23" t="n"/>
+      <c r="E61" s="21" t="n"/>
+      <c r="F61" s="22" t="n"/>
+      <c r="G61" s="23" t="n"/>
+      <c r="I61" s="21" t="n"/>
+      <c r="J61" s="22" t="n"/>
+      <c r="K61" s="23" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="13" t="inlineStr">
@@ -2953,50 +3067,50 @@
           <t>自營SP金額</t>
         </is>
       </c>
-      <c r="B63" s="13" t="n"/>
-      <c r="C63" s="13" t="n"/>
+      <c r="B63" s="17" t="n"/>
+      <c r="C63" s="18" t="n"/>
       <c r="E63" s="13" t="inlineStr">
         <is>
           <t>自營(SP增幅-BP增幅)金額</t>
         </is>
       </c>
-      <c r="F63" s="13" t="n"/>
-      <c r="G63" s="13" t="n"/>
+      <c r="F63" s="17" t="n"/>
+      <c r="G63" s="18" t="n"/>
       <c r="I63" s="13" t="inlineStr">
         <is>
           <t>自營BP/SP增幅比例</t>
         </is>
       </c>
-      <c r="J63" s="13" t="n"/>
-      <c r="K63" s="13" t="n"/>
+      <c r="J63" s="17" t="n"/>
+      <c r="K63" s="18" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="6" t="n">
         <v>208437</v>
       </c>
-      <c r="B64" s="6" t="n"/>
-      <c r="C64" s="6" t="n"/>
+      <c r="B64" s="19" t="n"/>
+      <c r="C64" s="20" t="n"/>
       <c r="E64" s="6" t="n">
         <v>7110</v>
       </c>
-      <c r="F64" s="6" t="n"/>
-      <c r="G64" s="6" t="n"/>
+      <c r="F64" s="19" t="n"/>
+      <c r="G64" s="20" t="n"/>
       <c r="I64" s="6" t="n">
         <v>0.01902284263959391</v>
       </c>
-      <c r="J64" s="6" t="n"/>
-      <c r="K64" s="6" t="n"/>
+      <c r="J64" s="19" t="n"/>
+      <c r="K64" s="20" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n"/>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="6" t="n"/>
-      <c r="E65" s="6" t="n"/>
-      <c r="F65" s="6" t="n"/>
-      <c r="G65" s="6" t="n"/>
-      <c r="I65" s="6" t="n"/>
-      <c r="J65" s="6" t="n"/>
-      <c r="K65" s="6" t="n"/>
+      <c r="A65" s="21" t="n"/>
+      <c r="B65" s="22" t="n"/>
+      <c r="C65" s="23" t="n"/>
+      <c r="E65" s="21" t="n"/>
+      <c r="F65" s="22" t="n"/>
+      <c r="G65" s="23" t="n"/>
+      <c r="I65" s="21" t="n"/>
+      <c r="J65" s="22" t="n"/>
+      <c r="K65" s="23" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3004,33 +3118,33 @@
           <t>仟元</t>
         </is>
       </c>
-      <c r="B66" s="7" t="n"/>
-      <c r="C66" s="7" t="n"/>
+      <c r="B66" s="19" t="n"/>
+      <c r="C66" s="20" t="n"/>
       <c r="E66" s="7" t="inlineStr">
         <is>
           <t>(208,437-216,317) - (242,314-257,304)</t>
         </is>
       </c>
-      <c r="F66" s="7" t="n"/>
-      <c r="G66" s="7" t="n"/>
+      <c r="F66" s="19" t="n"/>
+      <c r="G66" s="20" t="n"/>
       <c r="I66" s="7" t="inlineStr">
         <is>
           <t>(242,314-257,304) / (208,437-216,317) / 100</t>
         </is>
       </c>
-      <c r="J66" s="7" t="n"/>
-      <c r="K66" s="7" t="n"/>
+      <c r="J66" s="19" t="n"/>
+      <c r="K66" s="20" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="7" t="n"/>
-      <c r="B67" s="7" t="n"/>
-      <c r="C67" s="7" t="n"/>
-      <c r="E67" s="7" t="n"/>
-      <c r="F67" s="7" t="n"/>
-      <c r="G67" s="7" t="n"/>
-      <c r="I67" s="7" t="n"/>
-      <c r="J67" s="7" t="n"/>
-      <c r="K67" s="7" t="n"/>
+      <c r="A67" s="21" t="n"/>
+      <c r="B67" s="22" t="n"/>
+      <c r="C67" s="23" t="n"/>
+      <c r="E67" s="21" t="n"/>
+      <c r="F67" s="22" t="n"/>
+      <c r="G67" s="23" t="n"/>
+      <c r="I67" s="21" t="n"/>
+      <c r="J67" s="22" t="n"/>
+      <c r="K67" s="23" t="n"/>
     </row>
     <row r="78" ht="22" customHeight="1"/>
     <row r="96" ht="32" customHeight="1"/>

</xml_diff>

<commit_message>
Update chip report site 2026-05-18
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-04-22.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-04-22.xlsx
@@ -233,7 +233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -288,6 +288,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -686,7 +689,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -794,8 +796,6 @@
       <c r="J9" s="22" t="n"/>
       <c r="K9" s="23" t="n"/>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -987,7 +987,6 @@
       <c r="J23" s="22" t="n"/>
       <c r="K23" s="23" t="n"/>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
@@ -1073,7 +1072,6 @@
       <c r="J29" s="22" t="n"/>
       <c r="K29" s="23" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
@@ -1109,8 +1107,6 @@
       <c r="B35" s="22" t="n"/>
       <c r="C35" s="23" t="n"/>
     </row>
-    <row r="36"/>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
@@ -1302,7 +1298,6 @@
       <c r="J49" s="22" t="n"/>
       <c r="K49" s="23" t="n"/>
     </row>
-    <row r="50"/>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
@@ -1388,7 +1383,6 @@
       <c r="J55" s="22" t="n"/>
       <c r="K55" s="23" t="n"/>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
@@ -2229,6 +2223,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -2336,6 +2331,7 @@
       <c r="J9" s="22" t="n"/>
       <c r="K9" s="23" t="n"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
@@ -2421,6 +2417,8 @@
       <c r="J15" s="22" t="n"/>
       <c r="K15" s="23" t="n"/>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
@@ -2526,6 +2524,7 @@
       <c r="J23" s="22" t="n"/>
       <c r="K23" s="23" t="n"/>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
@@ -2560,7 +2559,7 @@
       </c>
       <c r="F26" s="19" t="n"/>
       <c r="G26" s="20" t="n"/>
-      <c r="I26" s="6" t="n">
+      <c r="I26" s="24" t="n">
         <v>0.3719298245614035</v>
       </c>
       <c r="J26" s="19" t="n"/>
@@ -2611,6 +2610,7 @@
       <c r="J29" s="22" t="n"/>
       <c r="K29" s="23" t="n"/>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
@@ -2696,6 +2696,7 @@
       <c r="J35" s="22" t="n"/>
       <c r="K35" s="23" t="n"/>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
@@ -2730,7 +2731,7 @@
       </c>
       <c r="F38" s="19" t="n"/>
       <c r="G38" s="20" t="n"/>
-      <c r="I38" s="6" t="n">
+      <c r="I38" s="24" t="n">
         <v>0.003620512292973974</v>
       </c>
       <c r="J38" s="19" t="n"/>
@@ -2781,6 +2782,8 @@
       <c r="J41" s="22" t="n"/>
       <c r="K41" s="23" t="n"/>
     </row>
+    <row r="42"/>
+    <row r="43"/>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="12" t="inlineStr">
         <is>
@@ -2886,6 +2889,7 @@
       <c r="J49" s="22" t="n"/>
       <c r="K49" s="23" t="n"/>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="13" t="inlineStr">
         <is>
@@ -2920,7 +2924,7 @@
       </c>
       <c r="F52" s="19" t="n"/>
       <c r="G52" s="20" t="n"/>
-      <c r="I52" s="6" t="n">
+      <c r="I52" s="24" t="n">
         <v>0.008166376536371788</v>
       </c>
       <c r="J52" s="19" t="n"/>
@@ -2971,6 +2975,7 @@
       <c r="J55" s="22" t="n"/>
       <c r="K55" s="23" t="n"/>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="13" t="inlineStr">
         <is>
@@ -3056,6 +3061,7 @@
       <c r="J61" s="22" t="n"/>
       <c r="K61" s="23" t="n"/>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="13" t="inlineStr">
         <is>
@@ -3090,7 +3096,7 @@
       </c>
       <c r="F64" s="19" t="n"/>
       <c r="G64" s="20" t="n"/>
-      <c r="I64" s="6" t="n">
+      <c r="I64" s="24" t="n">
         <v>0.01902284263959391</v>
       </c>
       <c r="J64" s="19" t="n"/>

</xml_diff>